<commit_message>
Polish submission: three presentation fixes for professor-facing deliverables
1. p-value display: bootstrap p-values that would print as exact 0.0 now
   render as "< 0.0001" in the Excel workbook (accurate upper bound from
   10,000 bootstrap reps; 0.0 is statistically improper).

2. 10_actuals_audit sheet: replaced the "(no data available)" fallback
   (which appeared because duplicate count = 0 leaves the duplicate-audit
   CSV empty) with a 13-row human-readable audit summary covering the
   IBES Actuals row count, ticker count, period, duplicates, anndats
   completeness, and both IBES tables + adjustment basis used.

3. 07_quality_checks.csv: cleaned "[np.int64(0), np.int64(1)]" debug
   artifact down to "[0, 1]" (Python 3.13 numpy-scalar repr leak);
   source script (09_quality_checks.py) patched so re-runs produce the
   clean output directly.

No pipeline changes; all numeric results unchanged.
</commit_message>
<xml_diff>
--- a/05_output/report/AUC_results_tables.xlsx
+++ b/05_output/report/AUC_results_tables.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="177">
   <si>
     <t>AUC of Analysts' Earnings Forecasts — Results Workbook</t>
   </si>
@@ -240,6 +240,9 @@
     <t>p_value_auc_le_0p5</t>
   </si>
   <si>
+    <t>&lt; 0.0001</t>
+  </si>
+  <si>
     <t>fyear</t>
   </si>
   <si>
@@ -375,9 +378,6 @@
     <t>lookahead=0, missing=0</t>
   </si>
   <si>
-    <t>[np.int64(0), np.int64(1)]</t>
-  </si>
-  <si>
     <t>[]</t>
   </si>
   <si>
@@ -438,7 +438,58 @@
     <t>AUC outside [0.45, 0.85] is unusual for analyst earnings forecast studies</t>
   </si>
   <si>
-    <t>(no data available)</t>
+    <t>audit_item</t>
+  </si>
+  <si>
+    <t>IBES Actuals: n rows</t>
+  </si>
+  <si>
+    <t>IBES Actuals: n unique tickers</t>
+  </si>
+  <si>
+    <t>IBES Actuals: period covered</t>
+  </si>
+  <si>
+    <t>Duplicate (ticker, fpedats) pairs</t>
+  </si>
+  <si>
+    <t>Rows with actual_anndats populated</t>
+  </si>
+  <si>
+    <t>% rows with actual_anndats</t>
+  </si>
+  <si>
+    <t>Duplicate audit rows exported</t>
+  </si>
+  <si>
+    <t>IBES Actuals table</t>
+  </si>
+  <si>
+    <t>IBES EPS basis (Actuals)</t>
+  </si>
+  <si>
+    <t>IBES Detail table</t>
+  </si>
+  <si>
+    <t>IBES EPS basis (Detail)</t>
+  </si>
+  <si>
+    <t>Overall audit</t>
+  </si>
+  <si>
+    <t>2004-12-31 → 2025-12-31</t>
+  </si>
+  <si>
+    <t>100.0%</t>
+  </si>
+  <si>
+    <t>ibes.act_epsus</t>
+  </si>
+  <si>
+    <t>ibes.det_epsus</t>
+  </si>
+  <si>
+    <t>PASS — 0 duplicates; matched adjusted basis for Actuals and Detail</t>
   </si>
   <si>
     <t>dataset</t>
@@ -1045,33 +1096,33 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E2" t="s">
         <v>124</v>
@@ -1079,16 +1130,16 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E3" t="s">
         <v>125</v>
@@ -1096,16 +1147,16 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E4" t="s">
         <v>126</v>
@@ -1113,16 +1164,16 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E5" t="s">
         <v>127</v>
@@ -1130,16 +1181,16 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E6" t="s">
         <v>127</v>
@@ -1147,16 +1198,16 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E7" t="s">
         <v>128</v>
@@ -1164,16 +1215,16 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E8" t="s">
         <v>129</v>
@@ -1181,16 +1232,16 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C9" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D9" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E9" t="s">
         <v>130</v>
@@ -1198,13 +1249,13 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D10" t="s">
         <v>120</v>
@@ -1215,13 +1266,13 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B11" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C11" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D11" t="s">
         <v>121</v>
@@ -1232,16 +1283,16 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B12" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C12" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D12" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E12" t="s">
         <v>133</v>
@@ -1249,10 +1300,10 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C13" t="s">
         <v>117</v>
@@ -1266,10 +1317,10 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C14" t="s">
         <v>118</v>
@@ -1283,10 +1334,10 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C15" t="s">
         <v>119</v>
@@ -1305,15 +1356,114 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" customWidth="1"/>
+    <col min="1" max="2" width="40.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" t="s">
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
         <v>137</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B2">
+        <v>65844</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>139</v>
+      </c>
+      <c r="B3">
+        <v>5757</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B4" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>141</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>142</v>
+      </c>
+      <c r="B6">
+        <v>65844</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>143</v>
+      </c>
+      <c r="B7" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>144</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>145</v>
+      </c>
+      <c r="B9" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>146</v>
+      </c>
+      <c r="B10" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>147</v>
+      </c>
+      <c r="B11" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>148</v>
+      </c>
+      <c r="B12" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>149</v>
+      </c>
+      <c r="B13" t="s">
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -1331,48 +1481,48 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
-        <v>138</v>
+        <v>155</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>139</v>
+        <v>156</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>141</v>
+        <v>158</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>142</v>
+        <v>159</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>143</v>
+        <v>160</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>144</v>
+        <v>161</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>145</v>
+        <v>162</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>146</v>
+        <v>163</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>147</v>
+        <v>164</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>148</v>
+        <v>165</v>
       </c>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>149</v>
+        <v>166</v>
       </c>
       <c r="B2" t="s">
-        <v>152</v>
+        <v>169</v>
       </c>
       <c r="C2" t="s">
-        <v>154</v>
+        <v>171</v>
       </c>
       <c r="D2">
         <v>37662</v>
@@ -1393,24 +1543,24 @@
         <v>5910</v>
       </c>
       <c r="J2" t="s">
-        <v>157</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>150</v>
+        <v>167</v>
       </c>
       <c r="B3" t="s">
-        <v>153</v>
+        <v>170</v>
       </c>
       <c r="C3" t="s">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="D3">
         <v>65844</v>
       </c>
       <c r="J3" t="s">
-        <v>158</v>
+        <v>175</v>
       </c>
       <c r="K3" t="s">
         <v>118</v>
@@ -1418,19 +1568,19 @@
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>151</v>
+        <v>168</v>
       </c>
       <c r="B4" t="s">
-        <v>153</v>
+        <v>170</v>
       </c>
       <c r="C4" t="s">
-        <v>156</v>
+        <v>173</v>
       </c>
       <c r="D4">
         <v>2301017</v>
       </c>
       <c r="J4" t="s">
-        <v>159</v>
+        <v>176</v>
       </c>
       <c r="K4" t="s">
         <v>118</v>
@@ -1802,8 +1952,8 @@
       <c r="Q2">
         <v>0.8135</v>
       </c>
-      <c r="R2">
-        <v>0</v>
+      <c r="R2" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1824,7 +1974,7 @@
         <v>39</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>41</v>
@@ -2657,7 +2807,7 @@
         <v>39</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>41</v>
@@ -2698,7 +2848,7 @@
         <v>48</v>
       </c>
       <c r="B2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C2">
         <v>6618</v>
@@ -2739,7 +2889,7 @@
         <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C3">
         <v>4182</v>
@@ -2780,7 +2930,7 @@
         <v>48</v>
       </c>
       <c r="B4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C4">
         <v>5576</v>
@@ -2821,7 +2971,7 @@
         <v>48</v>
       </c>
       <c r="B5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C5">
         <v>13089</v>
@@ -2859,10 +3009,10 @@
     </row>
     <row r="6" spans="1:13">
       <c r="A6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C6">
         <v>6618</v>
@@ -2900,10 +3050,10 @@
     </row>
     <row r="7" spans="1:13">
       <c r="A7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C7">
         <v>4182</v>
@@ -2941,10 +3091,10 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C8">
         <v>5576</v>
@@ -2982,10 +3132,10 @@
     </row>
     <row r="9" spans="1:13">
       <c r="A9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C9">
         <v>13089</v>
@@ -3023,10 +3173,10 @@
     </row>
     <row r="10" spans="1:13">
       <c r="A10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C10">
         <v>6618</v>
@@ -3064,10 +3214,10 @@
     </row>
     <row r="11" spans="1:13">
       <c r="A11" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B11" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C11">
         <v>4182</v>
@@ -3105,10 +3255,10 @@
     </row>
     <row r="12" spans="1:13">
       <c r="A12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C12">
         <v>5576</v>
@@ -3146,10 +3296,10 @@
     </row>
     <row r="13" spans="1:13">
       <c r="A13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C13">
         <v>13089</v>
@@ -3238,7 +3388,7 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B2">
         <v>29222</v>
@@ -3276,7 +3426,7 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B3">
         <v>29222</v>
@@ -3314,7 +3464,7 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B4">
         <v>29222</v>
@@ -3471,8 +3621,8 @@
       <c r="Q2">
         <v>0.8135</v>
       </c>
-      <c r="R2">
-        <v>0</v>
+      <c r="R2" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -3510,7 +3660,7 @@
         <v>0.6443577125403021</v>
       </c>
       <c r="L3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="M3">
         <v>10000</v>
@@ -3527,8 +3677,8 @@
       <c r="Q3">
         <v>0.8135</v>
       </c>
-      <c r="R3">
-        <v>0</v>
+      <c r="R3" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -3566,7 +3716,7 @@
         <v>0.6443577125403021</v>
       </c>
       <c r="L4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="M4">
         <v>10000</v>
@@ -3583,8 +3733,8 @@
       <c r="Q4">
         <v>0.8135</v>
       </c>
-      <c r="R4">
-        <v>0</v>
+      <c r="R4" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -3605,13 +3755,13 @@
         <v>39</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>41</v>
@@ -3652,7 +3802,7 @@
         <v>48</v>
       </c>
       <c r="B2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C2">
         <v>2005</v>
@@ -3699,7 +3849,7 @@
         <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C3">
         <v>2015</v>
@@ -3746,7 +3896,7 @@
         <v>48</v>
       </c>
       <c r="B4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C4">
         <v>2019</v>
@@ -3793,7 +3943,7 @@
         <v>48</v>
       </c>
       <c r="B5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C5">
         <v>2023</v>
@@ -3837,10 +3987,10 @@
     </row>
     <row r="6" spans="1:15">
       <c r="A6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C6">
         <v>2005</v>
@@ -3884,10 +4034,10 @@
     </row>
     <row r="7" spans="1:15">
       <c r="A7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C7">
         <v>2015</v>
@@ -3931,10 +4081,10 @@
     </row>
     <row r="8" spans="1:15">
       <c r="A8" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C8">
         <v>2019</v>
@@ -3978,10 +4128,10 @@
     </row>
     <row r="9" spans="1:15">
       <c r="A9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C9">
         <v>2023</v>
@@ -4025,10 +4175,10 @@
     </row>
     <row r="10" spans="1:15">
       <c r="A10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C10">
         <v>2005</v>
@@ -4072,10 +4222,10 @@
     </row>
     <row r="11" spans="1:15">
       <c r="A11" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C11">
         <v>2015</v>
@@ -4119,10 +4269,10 @@
     </row>
     <row r="12" spans="1:15">
       <c r="A12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C12">
         <v>2019</v>
@@ -4166,10 +4316,10 @@
     </row>
     <row r="13" spans="1:15">
       <c r="A13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C13">
         <v>2023</v>
@@ -4264,7 +4414,7 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B2">
         <v>29465</v>
@@ -4302,7 +4452,7 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B3">
         <v>29465</v>
@@ -4340,7 +4490,7 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B4">
         <v>29465</v>

</xml_diff>